<commit_message>
Fix VRES with ~0 MaxProd
</commit_message>
<xml_diff>
--- a/data/TX-123BT/Data_Sources.xlsx
+++ b/data/TX-123BT/Data_Sources.xlsx
@@ -852,7 +852,7 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>FuelCost=C1 [$/MWh], Efficiency=1, OMVarCost=0, CommitConsumption=C0/C1 [MWh/h] (C0 is a no-load cost per committed hour in the authors' SCUC despite its '$/MWh' label), StartupConsumption=Csu/C1 [MWh] - reproduces C1, C0 and Csu exactly in LEGO's cost terms; units with C1=0 (hydro) get 0 consumptions (their C0 and Csu are 0 as well); RampUp/RampDw=Ramping Rate [MW/min] × 60 [MW/h]; MinUpTime=MinDownTime=0 (not in the dataset; the authors' SCUC has no such constraint); EFOR, InertiaConst, CO2Emis left blank (not in the dataset); Hydro has no inflow data and is dispatched like a thermal unit (as in the authors' SCUC); g = 'G&lt;Gen Number&gt;_&lt;tec&gt;'. InvestCost (Coal, Natural Gas): InvestCost from Fraunhofer ISE 'Studie Stromgestehungskosten Erneuerbare Energien 2024', average of CAPEX min and max divided by lifetime (average of Steinkohle &amp; Braunkohle=Coal; Natural Gas=mean of Gas Turbine (OC Gas) and GuD (CC Gas), since TX-123BT does not distinguish them). Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
+          <t>FuelCost=C1 [$/MWh], Efficiency=1, OMVarCost=0, CommitConsumption=C0/C1 [MWh/h] (C0 is a no-load cost per committed hour in the authors' SCUC despite its '$/MWh' label), StartupConsumption=Csu/C1 [MWh] - reproduces C1, C0 and Csu exactly in LEGO's cost terms; units with C1=0 (hydro) get 0 consumptions (their C0 and Csu are 0 as well); RampUp/RampDw=Ramping Rate [MW/min] × 60 [MW/h]; MinUpTime=MinDownTime=1 h (not in the dataset, the authors' SCUC has no such constraint; 1 h is the floor for every unit); EFOR, InertiaConst, CO2Emis left blank (not in the dataset); Hydro has no inflow data and is dispatched like a thermal unit (as in the authors' SCUC); g = 'G&lt;Gen Number&gt;_&lt;tec&gt;'. InvestCost (Coal, Natural Gas): InvestCost from Fraunhofer ISE 'Studie Stromgestehungskosten Erneuerbare Energien 2024', average of CAPEX min and max divided by lifetime (average of Steinkohle &amp; Braunkohle=Coal; Natural Gas=mean of Gas Turbine (OC Gas) and GuD (CC Gas), since TX-123BT does not distinguish them). Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>FuelCost=C1 [$/MWh], Efficiency=1, OMVarCost=0, CommitConsumption=C0/C1 [MWh/h] (C0 is a no-load cost per committed hour in the authors' SCUC despite its '$/MWh' label), StartupConsumption=Csu/C1 [MWh] - reproduces C1, C0 and Csu exactly in LEGO's cost terms; units with C1=0 (hydro) get 0 consumptions (their C0 and Csu are 0 as well); RampUp/RampDw=Ramping Rate [MW/min] × 60 [MW/h]; MinUpTime=MinDownTime=0 (not in the dataset; the authors' SCUC has no such constraint); EFOR, InertiaConst, CO2Emis left blank (not in the dataset); Hydro has no inflow data and is dispatched like a thermal unit (as in the authors' SCUC); g = 'G&lt;Gen Number&gt;_&lt;tec&gt;'. InvestCost (Hydro): InvestCost from dena Leitstudie Integrierte Energiewende 2018, Kosten 2020 for Speicherwasser divided by lifetime. Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
+          <t>FuelCost=C1 [$/MWh], Efficiency=1, OMVarCost=0, CommitConsumption=C0/C1 [MWh/h] (C0 is a no-load cost per committed hour in the authors' SCUC despite its '$/MWh' label), StartupConsumption=Csu/C1 [MWh] - reproduces C1, C0 and Csu exactly in LEGO's cost terms; units with C1=0 (hydro) get 0 consumptions (their C0 and Csu are 0 as well); RampUp/RampDw=Ramping Rate [MW/min] × 60 [MW/h]; MinUpTime=MinDownTime=1 h (not in the dataset, the authors' SCUC has no such constraint; 1 h is the floor for every unit); EFOR, InertiaConst, CO2Emis left blank (not in the dataset); Hydro has no inflow data and is dispatched like a thermal unit (as in the authors' SCUC); g = 'G&lt;Gen Number&gt;_&lt;tec&gt;'. InvestCost (Hydro): InvestCost from dena Leitstudie Integrierte Energiewende 2018, Kosten 2020 for Speicherwasser divided by lifetime. Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>FuelCost=C1 [$/MWh], Efficiency=1, OMVarCost=0, CommitConsumption=C0/C1 [MWh/h] (C0 is a no-load cost per committed hour in the authors' SCUC despite its '$/MWh' label), StartupConsumption=Csu/C1 [MWh] - reproduces C1, C0 and Csu exactly in LEGO's cost terms; units with C1=0 (hydro) get 0 consumptions (their C0 and Csu are 0 as well); RampUp/RampDw=Ramping Rate [MW/min] × 60 [MW/h]; MinUpTime=MinDownTime=0 (not in the dataset; the authors' SCUC has no such constraint); EFOR, InertiaConst, CO2Emis left blank (not in the dataset); Hydro has no inflow data and is dispatched like a thermal unit (as in the authors' SCUC); g = 'G&lt;Gen Number&gt;_&lt;tec&gt;'. InvestCost (Nuclear): Placeholder investment cost - can be updated in future with real-world cost. Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
+          <t>FuelCost=C1 [$/MWh], Efficiency=1, OMVarCost=0, CommitConsumption=C0/C1 [MWh/h] (C0 is a no-load cost per committed hour in the authors' SCUC despite its '$/MWh' label), StartupConsumption=Csu/C1 [MWh] - reproduces C1, C0 and Csu exactly in LEGO's cost terms; units with C1=0 (hydro) get 0 consumptions (their C0 and Csu are 0 as well); RampUp/RampDw=Ramping Rate [MW/min] × 60 [MW/h]; MinUpTime=MinDownTime=1 h (not in the dataset, the authors' SCUC has no such constraint; 1 h is the floor for every unit); EFOR, InertiaConst, CO2Emis left blank (not in the dataset); Hydro has no inflow data and is dispatched like a thermal unit (as in the authors' SCUC); g = 'G&lt;Gen Number&gt;_&lt;tec&gt;'. InvestCost (Nuclear): Placeholder investment cost - can be updated in future with real-world cost. Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>MaxProd=max(Pmax, peak of the Wind_5y/Solar_5y profiles over all translated years): every solar profile exceeds its Pmax by 8-27 %, and the authors' SCUC uses the profile MW unclipped; wind stays within Pmax; OMVarCost=C1 (0 for all); g = 'G&lt;Gen Number&gt;_&lt;tec&gt;'. InvestCost (Wind, Solar): InvestCost for Wind and Solar from Fraunhofer ISE 'Studie Stromgestehungskosten Erneuerbare Energien 2024', average of min/max divided by lifetime. Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
+          <t>MaxProd=max(Pmax, peak of the Wind_5y/Solar_5y profiles over all translated years): every solar profile exceeds its Pmax by 8-27 %, and the authors' SCUC uses the profile MW unclipped; wind stays within Pmax; OMVarCost=C1 (0 for all); EnableInvest=0 for plants without output in any translated year (for 2017-2021 the wind plants G84, G134, G159, G169, whose Pmax is ~1e-5 MW), so with ExisUnits=0 their capacity is 0; g = 'G&lt;Gen Number&gt;_&lt;tec&gt;'. InvestCost (Wind, Solar): InvestCost for Wind and Solar from Fraunhofer ISE 'Studie Stromgestehungskosten Erneuerbare Energien 2024', average of min/max divided by lifetime. Per-generator ±0.5 % deterministic variation applied to prevent degenerate optimisation.</t>
         </is>
       </c>
     </row>

</xml_diff>